<commit_message>
Update pattern tracker: 16 issues by category in 'How to use', add Category column to tracker
</commit_message>
<xml_diff>
--- a/pattern-tracker.xlsx
+++ b/pattern-tracker.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="9">
+  <fonts count="12">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -71,6 +71,17 @@
       <color rgb="0001696F"/>
       <sz val="12"/>
     </font>
+    <font>
+      <b val="1"/>
+      <sz val="12"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <i val="1"/>
+    </font>
+    <font>
+      <b val="1"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -111,7 +122,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="13">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -137,6 +148,14 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -502,7 +521,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A32"/>
+  <dimension ref="A1:A54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -633,82 +652,200 @@
       <c r="A20" s="3" t="inlineStr"/>
     </row>
     <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>The 8 issues seeded in the repo</t>
+      <c r="A21" s="9" t="inlineStr">
+        <is>
+          <t>The 16 issues seeded in the repo (organized by category)</t>
         </is>
       </c>
     </row>
     <row r="22">
-      <c r="A22" s="3" t="inlineStr">
-        <is>
-          <t>#1  index.md — Add structure and a real 'What is Quillship?' section  (good first issue)</t>
+      <c r="A22" s="10" t="inlineStr">
+        <is>
+          <t>Top level</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="3" t="inlineStr">
         <is>
-          <t>#2  getting-started.md — Tag code blocks, add prerequisites  (good first issue)</t>
+          <t xml:space="preserve">  #1  index.md — Add structure and a real 'What is Quillship?' section  (good first issue)</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="3" t="inlineStr">
         <is>
-          <t>#3  api-reference.md — Break the wall of prose into structured endpoints</t>
+          <t xml:space="preserve">  #2  getting-started.md — Tag code blocks, add prerequisites  (good first issue)</t>
         </is>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="3" t="inlineStr">
         <is>
-          <t>#4  authentication.md — Name the header, show a real example</t>
+          <t xml:space="preserve">  #3  api-reference.md — Break wall of prose into structured endpoints (Path C / scope-down option in issue body)</t>
         </is>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="3" t="inlineStr">
         <is>
-          <t>#5  webhooks.md — Fix broken anchors, define acronyms, add payload example</t>
+          <t xml:space="preserve">  #4  authentication.md — Name the header, show a real example</t>
         </is>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="3" t="inlineStr">
         <is>
-          <t>#6  sdks/python.md — Add install command, tag python code blocks  (good first issue)</t>
+          <t xml:space="preserve">  #5  webhooks.md — Fix broken anchors, define acronyms, add payload example</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="3" t="inlineStr">
         <is>
-          <t>#7  migrate-from-wordpress.md — Break the 3KB paragraph into ordered steps</t>
+          <t xml:space="preserve">  #8  faq.md — Replace circular answers with real ones, add llms.txt</t>
         </is>
       </c>
     </row>
     <row r="29">
-      <c r="A29" s="3" t="inlineStr">
-        <is>
-          <t>#8  faq.md — Replace circular answers with real ones, add llms.txt</t>
-        </is>
-      </c>
+      <c r="A29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="3" t="inlineStr"/>
+      <c r="A30" s="10" t="inlineStr">
+        <is>
+          <t>Concepts</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
+          <t xml:space="preserve">  #9  concepts/content-model.md — Replace abstract prose with concrete schema example</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="n"/>
+    </row>
+    <row r="33">
+      <c r="A33" s="11" t="inlineStr">
+        <is>
+          <t>API</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #10  api/graphql.md — Show actual queries and schema</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #11  api/rate-limits.md — Move numbers from prose into a table  (good first issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36"/>
+    <row r="37">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
+          <t>SDKs</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #6  sdks/python.md — Add install command, tag python code blocks  (good first issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #12  sdks/javascript.md — Fix import, add language tags, strengthen TS section  (good first issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="40"/>
+    <row r="41">
+      <c r="A41" s="11" t="inlineStr">
+        <is>
+          <t>Guides</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #7  guides/migrate-from-wordpress.md — Break 3KB paragraph into ordered steps</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #13  guides/quickstart-react.md — Add prerequisites, slow down advanced jumps</t>
+        </is>
+      </c>
+    </row>
+    <row r="44"/>
+    <row r="45">
+      <c r="A45" s="11" t="inlineStr">
+        <is>
+          <t>Operations</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #14  ops/deployment.md — Replace generic guidance with concrete env vars and example</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="11" t="inlineStr">
+        <is>
+          <t>Reference</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #15  reference/cli.md — Add flags, args, and examples to commands</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #16  reference/glossary.md — Replace tautological definitions with real ones  (good first issue)</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" t="inlineStr">
+        <is>
           <t>Repo: https://github.com/wtd-quillship-demo/quillship-docs</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="5" t="inlineStr">
+    <row r="53">
+      <c r="A53" t="inlineStr">
         <is>
           <t>Live site to audit: https://wtd-quillship-demo.github.io/quillship-docs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" t="inlineStr">
+        <is>
+          <t>Canonical fix criteria: https://github.com/wtd-quillship-demo/quillship-docs/blob/main/CONTRIBUTING.md#what-ai-readiness-means-here-canonical-list</t>
         </is>
       </c>
     </row>
@@ -723,19 +860,20 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J63"/>
+  <dimension ref="A1:K63"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="38" customWidth="1" min="2" max="2"/>
-    <col width="9" customWidth="1" min="3" max="3"/>
-    <col width="42" customWidth="1" min="4" max="4"/>
-    <col width="11" customWidth="1" min="5" max="5"/>
-    <col width="50" customWidth="1" min="6" max="6"/>
-    <col width="13" customWidth="1" min="7" max="7"/>
-    <col width="12" customWidth="1" min="8" max="8"/>
-    <col width="11" customWidth="1" min="9" max="9"/>
-    <col width="36" customWidth="1" min="10" max="10"/>
+    <col width="32" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="40" customWidth="1" min="5" max="5"/>
+    <col width="10" customWidth="1" min="6" max="6"/>
+    <col width="38" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="35" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="32" customHeight="1">
@@ -749,42 +887,47 @@
           <t>Site or File</t>
         </is>
       </c>
-      <c r="C1" s="6" t="inlineStr">
+      <c r="C1" s="12" t="inlineStr">
+        <is>
+          <t>Category</t>
+        </is>
+      </c>
+      <c r="D1" s="6" t="inlineStr">
         <is>
           <t>Issue #</t>
         </is>
       </c>
-      <c r="D1" s="6" t="inlineStr">
+      <c r="E1" s="6" t="inlineStr">
         <is>
           <t>Anti-Pattern Spotted</t>
         </is>
       </c>
-      <c r="E1" s="6" t="inlineStr">
+      <c r="F1" s="6" t="inlineStr">
         <is>
           <t>Severity</t>
         </is>
       </c>
-      <c r="F1" s="6" t="inlineStr">
+      <c r="G1" s="6" t="inlineStr">
         <is>
           <t>Fix Applied</t>
         </is>
       </c>
-      <c r="G1" s="6" t="inlineStr">
+      <c r="H1" s="6" t="inlineStr">
         <is>
           <t>Score Before</t>
         </is>
       </c>
-      <c r="H1" s="6" t="inlineStr">
+      <c r="I1" s="6" t="inlineStr">
         <is>
           <t>Score After</t>
         </is>
       </c>
-      <c r="I1" s="6" t="inlineStr">
+      <c r="J1" s="6" t="inlineStr">
         <is>
           <t>Score Delta</t>
         </is>
       </c>
-      <c r="J1" s="6" t="inlineStr">
+      <c r="K1" s="6" t="inlineStr">
         <is>
           <t>Notes</t>
         </is>
@@ -801,35 +944,40 @@
           <t>docs/api-reference.md</t>
         </is>
       </c>
-      <c r="C2" s="7" t="n">
+      <c r="C2" t="inlineStr">
+        <is>
+          <t>Top level</t>
+        </is>
+      </c>
+      <c r="D2" s="7" t="n">
         <v>3</v>
       </c>
-      <c r="D2" s="7" t="inlineStr">
+      <c r="E2" s="7" t="inlineStr">
         <is>
           <t>Wall of prose, no endpoint headings</t>
         </is>
       </c>
-      <c r="E2" s="7" t="inlineStr">
+      <c r="F2" s="7" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="F2" s="7" t="inlineStr">
+      <c r="G2" s="7" t="inlineStr">
         <is>
           <t>Split into H2 per endpoint with request/response example each</t>
         </is>
       </c>
-      <c r="G2" s="7" t="n">
+      <c r="H2" s="7" t="n">
         <v>42</v>
       </c>
-      <c r="H2" s="7" t="n">
+      <c r="I2" s="7" t="n">
         <v>71</v>
       </c>
-      <c r="I2" s="7">
-        <f>H2-G2</f>
-        <v/>
-      </c>
-      <c r="J2" s="7" t="inlineStr">
+      <c r="J2" s="7">
+        <f>I2-H2</f>
+        <v/>
+      </c>
+      <c r="K2" s="7" t="inlineStr">
         <is>
           <t>LLM could now answer 'how do I delete content' correctly</t>
         </is>
@@ -846,37 +994,42 @@
           <t>docs.your-real-site.com</t>
         </is>
       </c>
-      <c r="C3" s="7" t="inlineStr">
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>External</t>
+        </is>
+      </c>
+      <c r="D3" s="7" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="D3" s="7" t="inlineStr">
+      <c r="E3" s="7" t="inlineStr">
         <is>
           <t>Code blocks with no language tag</t>
         </is>
       </c>
-      <c r="E3" s="7" t="inlineStr">
+      <c r="F3" s="7" t="inlineStr">
         <is>
           <t>Med</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
+      <c r="G3" s="7" t="inlineStr">
         <is>
           <t>Added language tags to 12 code samples</t>
         </is>
       </c>
-      <c r="G3" s="7" t="n">
+      <c r="H3" s="7" t="n">
         <v>58</v>
       </c>
-      <c r="H3" s="7" t="n">
+      <c r="I3" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="I3" s="7">
-        <f>H3-G3</f>
-        <v/>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
+      <c r="J3" s="7">
+        <f>I3-H3</f>
+        <v/>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
         <is>
           <t>Stripe-style format</t>
         </is>
@@ -885,906 +1038,912 @@
     <row r="4">
       <c r="A4" s="8" t="n"/>
       <c r="B4" s="8" t="n"/>
-      <c r="C4" s="8" t="n"/>
       <c r="D4" s="8" t="n"/>
       <c r="E4" s="8" t="n"/>
       <c r="F4" s="8" t="n"/>
       <c r="G4" s="8" t="n"/>
       <c r="H4" s="8" t="n"/>
-      <c r="I4" s="8">
-        <f>IF(AND(ISNUMBER(G4),ISNUMBER(H4)),H4-G4,"")</f>
-        <v/>
-      </c>
-      <c r="J4" s="8" t="n"/>
+      <c r="I4" s="8" t="n"/>
+      <c r="J4" s="8">
+        <f>IF(AND(ISNUMBER(H4),ISNUMBER(I4)),I4-H4,"")</f>
+        <v/>
+      </c>
+      <c r="K4" s="8" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="8" t="n"/>
       <c r="B5" s="8" t="n"/>
-      <c r="C5" s="8" t="n"/>
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="8" t="n"/>
       <c r="F5" s="8" t="n"/>
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
-      <c r="I5" s="8">
-        <f>IF(AND(ISNUMBER(G5),ISNUMBER(H5)),H5-G5,"")</f>
-        <v/>
-      </c>
-      <c r="J5" s="8" t="n"/>
+      <c r="I5" s="8" t="n"/>
+      <c r="J5" s="8">
+        <f>IF(AND(ISNUMBER(H5),ISNUMBER(I5)),I5-H5,"")</f>
+        <v/>
+      </c>
+      <c r="K5" s="8" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="8" t="n"/>
       <c r="B6" s="8" t="n"/>
-      <c r="C6" s="8" t="n"/>
       <c r="D6" s="8" t="n"/>
       <c r="E6" s="8" t="n"/>
       <c r="F6" s="8" t="n"/>
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="8" t="n"/>
-      <c r="I6" s="8">
-        <f>IF(AND(ISNUMBER(G6),ISNUMBER(H6)),H6-G6,"")</f>
-        <v/>
-      </c>
-      <c r="J6" s="8" t="n"/>
+      <c r="I6" s="8" t="n"/>
+      <c r="J6" s="8">
+        <f>IF(AND(ISNUMBER(H6),ISNUMBER(I6)),I6-H6,"")</f>
+        <v/>
+      </c>
+      <c r="K6" s="8" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="8" t="n"/>
       <c r="B7" s="8" t="n"/>
-      <c r="C7" s="8" t="n"/>
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="8" t="n"/>
       <c r="F7" s="8" t="n"/>
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="8" t="n"/>
-      <c r="I7" s="8">
-        <f>IF(AND(ISNUMBER(G7),ISNUMBER(H7)),H7-G7,"")</f>
-        <v/>
-      </c>
-      <c r="J7" s="8" t="n"/>
+      <c r="I7" s="8" t="n"/>
+      <c r="J7" s="8">
+        <f>IF(AND(ISNUMBER(H7),ISNUMBER(I7)),I7-H7,"")</f>
+        <v/>
+      </c>
+      <c r="K7" s="8" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="8" t="n"/>
       <c r="B8" s="8" t="n"/>
-      <c r="C8" s="8" t="n"/>
       <c r="D8" s="8" t="n"/>
       <c r="E8" s="8" t="n"/>
       <c r="F8" s="8" t="n"/>
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="8" t="n"/>
-      <c r="I8" s="8">
-        <f>IF(AND(ISNUMBER(G8),ISNUMBER(H8)),H8-G8,"")</f>
-        <v/>
-      </c>
-      <c r="J8" s="8" t="n"/>
+      <c r="I8" s="8" t="n"/>
+      <c r="J8" s="8">
+        <f>IF(AND(ISNUMBER(H8),ISNUMBER(I8)),I8-H8,"")</f>
+        <v/>
+      </c>
+      <c r="K8" s="8" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="8" t="n"/>
       <c r="B9" s="8" t="n"/>
-      <c r="C9" s="8" t="n"/>
       <c r="D9" s="8" t="n"/>
       <c r="E9" s="8" t="n"/>
       <c r="F9" s="8" t="n"/>
       <c r="G9" s="8" t="n"/>
       <c r="H9" s="8" t="n"/>
-      <c r="I9" s="8">
-        <f>IF(AND(ISNUMBER(G9),ISNUMBER(H9)),H9-G9,"")</f>
-        <v/>
-      </c>
-      <c r="J9" s="8" t="n"/>
+      <c r="I9" s="8" t="n"/>
+      <c r="J9" s="8">
+        <f>IF(AND(ISNUMBER(H9),ISNUMBER(I9)),I9-H9,"")</f>
+        <v/>
+      </c>
+      <c r="K9" s="8" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="8" t="n"/>
       <c r="B10" s="8" t="n"/>
-      <c r="C10" s="8" t="n"/>
       <c r="D10" s="8" t="n"/>
       <c r="E10" s="8" t="n"/>
       <c r="F10" s="8" t="n"/>
       <c r="G10" s="8" t="n"/>
       <c r="H10" s="8" t="n"/>
-      <c r="I10" s="8">
-        <f>IF(AND(ISNUMBER(G10),ISNUMBER(H10)),H10-G10,"")</f>
-        <v/>
-      </c>
-      <c r="J10" s="8" t="n"/>
+      <c r="I10" s="8" t="n"/>
+      <c r="J10" s="8">
+        <f>IF(AND(ISNUMBER(H10),ISNUMBER(I10)),I10-H10,"")</f>
+        <v/>
+      </c>
+      <c r="K10" s="8" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="8" t="n"/>
       <c r="B11" s="8" t="n"/>
-      <c r="C11" s="8" t="n"/>
       <c r="D11" s="8" t="n"/>
       <c r="E11" s="8" t="n"/>
       <c r="F11" s="8" t="n"/>
       <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
-      <c r="I11" s="8">
-        <f>IF(AND(ISNUMBER(G11),ISNUMBER(H11)),H11-G11,"")</f>
-        <v/>
-      </c>
-      <c r="J11" s="8" t="n"/>
+      <c r="I11" s="8" t="n"/>
+      <c r="J11" s="8">
+        <f>IF(AND(ISNUMBER(H11),ISNUMBER(I11)),I11-H11,"")</f>
+        <v/>
+      </c>
+      <c r="K11" s="8" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="8" t="n"/>
       <c r="B12" s="8" t="n"/>
-      <c r="C12" s="8" t="n"/>
       <c r="D12" s="8" t="n"/>
       <c r="E12" s="8" t="n"/>
       <c r="F12" s="8" t="n"/>
       <c r="G12" s="8" t="n"/>
       <c r="H12" s="8" t="n"/>
-      <c r="I12" s="8">
-        <f>IF(AND(ISNUMBER(G12),ISNUMBER(H12)),H12-G12,"")</f>
-        <v/>
-      </c>
-      <c r="J12" s="8" t="n"/>
+      <c r="I12" s="8" t="n"/>
+      <c r="J12" s="8">
+        <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12)),I12-H12,"")</f>
+        <v/>
+      </c>
+      <c r="K12" s="8" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="8" t="n"/>
       <c r="B13" s="8" t="n"/>
-      <c r="C13" s="8" t="n"/>
       <c r="D13" s="8" t="n"/>
       <c r="E13" s="8" t="n"/>
       <c r="F13" s="8" t="n"/>
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
-      <c r="I13" s="8">
-        <f>IF(AND(ISNUMBER(G13),ISNUMBER(H13)),H13-G13,"")</f>
-        <v/>
-      </c>
-      <c r="J13" s="8" t="n"/>
+      <c r="I13" s="8" t="n"/>
+      <c r="J13" s="8">
+        <f>IF(AND(ISNUMBER(H13),ISNUMBER(I13)),I13-H13,"")</f>
+        <v/>
+      </c>
+      <c r="K13" s="8" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="8" t="n"/>
       <c r="B14" s="8" t="n"/>
-      <c r="C14" s="8" t="n"/>
       <c r="D14" s="8" t="n"/>
       <c r="E14" s="8" t="n"/>
       <c r="F14" s="8" t="n"/>
       <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
-      <c r="I14" s="8">
-        <f>IF(AND(ISNUMBER(G14),ISNUMBER(H14)),H14-G14,"")</f>
-        <v/>
-      </c>
-      <c r="J14" s="8" t="n"/>
+      <c r="I14" s="8" t="n"/>
+      <c r="J14" s="8">
+        <f>IF(AND(ISNUMBER(H14),ISNUMBER(I14)),I14-H14,"")</f>
+        <v/>
+      </c>
+      <c r="K14" s="8" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="8" t="n"/>
       <c r="B15" s="8" t="n"/>
-      <c r="C15" s="8" t="n"/>
       <c r="D15" s="8" t="n"/>
       <c r="E15" s="8" t="n"/>
       <c r="F15" s="8" t="n"/>
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
-      <c r="I15" s="8">
-        <f>IF(AND(ISNUMBER(G15),ISNUMBER(H15)),H15-G15,"")</f>
-        <v/>
-      </c>
-      <c r="J15" s="8" t="n"/>
+      <c r="I15" s="8" t="n"/>
+      <c r="J15" s="8">
+        <f>IF(AND(ISNUMBER(H15),ISNUMBER(I15)),I15-H15,"")</f>
+        <v/>
+      </c>
+      <c r="K15" s="8" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="8" t="n"/>
       <c r="B16" s="8" t="n"/>
-      <c r="C16" s="8" t="n"/>
       <c r="D16" s="8" t="n"/>
       <c r="E16" s="8" t="n"/>
       <c r="F16" s="8" t="n"/>
       <c r="G16" s="8" t="n"/>
       <c r="H16" s="8" t="n"/>
-      <c r="I16" s="8">
-        <f>IF(AND(ISNUMBER(G16),ISNUMBER(H16)),H16-G16,"")</f>
-        <v/>
-      </c>
-      <c r="J16" s="8" t="n"/>
+      <c r="I16" s="8" t="n"/>
+      <c r="J16" s="8">
+        <f>IF(AND(ISNUMBER(H16),ISNUMBER(I16)),I16-H16,"")</f>
+        <v/>
+      </c>
+      <c r="K16" s="8" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="8" t="n"/>
       <c r="B17" s="8" t="n"/>
-      <c r="C17" s="8" t="n"/>
       <c r="D17" s="8" t="n"/>
       <c r="E17" s="8" t="n"/>
       <c r="F17" s="8" t="n"/>
       <c r="G17" s="8" t="n"/>
       <c r="H17" s="8" t="n"/>
-      <c r="I17" s="8">
-        <f>IF(AND(ISNUMBER(G17),ISNUMBER(H17)),H17-G17,"")</f>
-        <v/>
-      </c>
-      <c r="J17" s="8" t="n"/>
+      <c r="I17" s="8" t="n"/>
+      <c r="J17" s="8">
+        <f>IF(AND(ISNUMBER(H17),ISNUMBER(I17)),I17-H17,"")</f>
+        <v/>
+      </c>
+      <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="8" t="n"/>
       <c r="B18" s="8" t="n"/>
-      <c r="C18" s="8" t="n"/>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="8" t="n"/>
       <c r="F18" s="8" t="n"/>
       <c r="G18" s="8" t="n"/>
       <c r="H18" s="8" t="n"/>
-      <c r="I18" s="8">
-        <f>IF(AND(ISNUMBER(G18),ISNUMBER(H18)),H18-G18,"")</f>
-        <v/>
-      </c>
-      <c r="J18" s="8" t="n"/>
+      <c r="I18" s="8" t="n"/>
+      <c r="J18" s="8">
+        <f>IF(AND(ISNUMBER(H18),ISNUMBER(I18)),I18-H18,"")</f>
+        <v/>
+      </c>
+      <c r="K18" s="8" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="8" t="n"/>
       <c r="B19" s="8" t="n"/>
-      <c r="C19" s="8" t="n"/>
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="8" t="n"/>
       <c r="F19" s="8" t="n"/>
       <c r="G19" s="8" t="n"/>
       <c r="H19" s="8" t="n"/>
-      <c r="I19" s="8">
-        <f>IF(AND(ISNUMBER(G19),ISNUMBER(H19)),H19-G19,"")</f>
-        <v/>
-      </c>
-      <c r="J19" s="8" t="n"/>
+      <c r="I19" s="8" t="n"/>
+      <c r="J19" s="8">
+        <f>IF(AND(ISNUMBER(H19),ISNUMBER(I19)),I19-H19,"")</f>
+        <v/>
+      </c>
+      <c r="K19" s="8" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="8" t="n"/>
       <c r="B20" s="8" t="n"/>
-      <c r="C20" s="8" t="n"/>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="8" t="n"/>
       <c r="F20" s="8" t="n"/>
       <c r="G20" s="8" t="n"/>
       <c r="H20" s="8" t="n"/>
-      <c r="I20" s="8">
-        <f>IF(AND(ISNUMBER(G20),ISNUMBER(H20)),H20-G20,"")</f>
-        <v/>
-      </c>
-      <c r="J20" s="8" t="n"/>
+      <c r="I20" s="8" t="n"/>
+      <c r="J20" s="8">
+        <f>IF(AND(ISNUMBER(H20),ISNUMBER(I20)),I20-H20,"")</f>
+        <v/>
+      </c>
+      <c r="K20" s="8" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="8" t="n"/>
       <c r="B21" s="8" t="n"/>
-      <c r="C21" s="8" t="n"/>
       <c r="D21" s="8" t="n"/>
       <c r="E21" s="8" t="n"/>
       <c r="F21" s="8" t="n"/>
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
-      <c r="I21" s="8">
-        <f>IF(AND(ISNUMBER(G21),ISNUMBER(H21)),H21-G21,"")</f>
-        <v/>
-      </c>
-      <c r="J21" s="8" t="n"/>
+      <c r="I21" s="8" t="n"/>
+      <c r="J21" s="8">
+        <f>IF(AND(ISNUMBER(H21),ISNUMBER(I21)),I21-H21,"")</f>
+        <v/>
+      </c>
+      <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="8" t="n"/>
       <c r="B22" s="8" t="n"/>
-      <c r="C22" s="8" t="n"/>
       <c r="D22" s="8" t="n"/>
       <c r="E22" s="8" t="n"/>
       <c r="F22" s="8" t="n"/>
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
-      <c r="I22" s="8">
-        <f>IF(AND(ISNUMBER(G22),ISNUMBER(H22)),H22-G22,"")</f>
-        <v/>
-      </c>
-      <c r="J22" s="8" t="n"/>
+      <c r="I22" s="8" t="n"/>
+      <c r="J22" s="8">
+        <f>IF(AND(ISNUMBER(H22),ISNUMBER(I22)),I22-H22,"")</f>
+        <v/>
+      </c>
+      <c r="K22" s="8" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="8" t="n"/>
       <c r="B23" s="8" t="n"/>
-      <c r="C23" s="8" t="n"/>
       <c r="D23" s="8" t="n"/>
       <c r="E23" s="8" t="n"/>
       <c r="F23" s="8" t="n"/>
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
-      <c r="I23" s="8">
-        <f>IF(AND(ISNUMBER(G23),ISNUMBER(H23)),H23-G23,"")</f>
-        <v/>
-      </c>
-      <c r="J23" s="8" t="n"/>
+      <c r="I23" s="8" t="n"/>
+      <c r="J23" s="8">
+        <f>IF(AND(ISNUMBER(H23),ISNUMBER(I23)),I23-H23,"")</f>
+        <v/>
+      </c>
+      <c r="K23" s="8" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="8" t="n"/>
       <c r="B24" s="8" t="n"/>
-      <c r="C24" s="8" t="n"/>
       <c r="D24" s="8" t="n"/>
       <c r="E24" s="8" t="n"/>
       <c r="F24" s="8" t="n"/>
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
-      <c r="I24" s="8">
-        <f>IF(AND(ISNUMBER(G24),ISNUMBER(H24)),H24-G24,"")</f>
-        <v/>
-      </c>
-      <c r="J24" s="8" t="n"/>
+      <c r="I24" s="8" t="n"/>
+      <c r="J24" s="8">
+        <f>IF(AND(ISNUMBER(H24),ISNUMBER(I24)),I24-H24,"")</f>
+        <v/>
+      </c>
+      <c r="K24" s="8" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="8" t="n"/>
       <c r="B25" s="8" t="n"/>
-      <c r="C25" s="8" t="n"/>
       <c r="D25" s="8" t="n"/>
       <c r="E25" s="8" t="n"/>
       <c r="F25" s="8" t="n"/>
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
-      <c r="I25" s="8">
-        <f>IF(AND(ISNUMBER(G25),ISNUMBER(H25)),H25-G25,"")</f>
-        <v/>
-      </c>
-      <c r="J25" s="8" t="n"/>
+      <c r="I25" s="8" t="n"/>
+      <c r="J25" s="8">
+        <f>IF(AND(ISNUMBER(H25),ISNUMBER(I25)),I25-H25,"")</f>
+        <v/>
+      </c>
+      <c r="K25" s="8" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="8" t="n"/>
       <c r="B26" s="8" t="n"/>
-      <c r="C26" s="8" t="n"/>
       <c r="D26" s="8" t="n"/>
       <c r="E26" s="8" t="n"/>
       <c r="F26" s="8" t="n"/>
       <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
-      <c r="I26" s="8">
-        <f>IF(AND(ISNUMBER(G26),ISNUMBER(H26)),H26-G26,"")</f>
-        <v/>
-      </c>
-      <c r="J26" s="8" t="n"/>
+      <c r="I26" s="8" t="n"/>
+      <c r="J26" s="8">
+        <f>IF(AND(ISNUMBER(H26),ISNUMBER(I26)),I26-H26,"")</f>
+        <v/>
+      </c>
+      <c r="K26" s="8" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="8" t="n"/>
       <c r="B27" s="8" t="n"/>
-      <c r="C27" s="8" t="n"/>
       <c r="D27" s="8" t="n"/>
       <c r="E27" s="8" t="n"/>
       <c r="F27" s="8" t="n"/>
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
-      <c r="I27" s="8">
-        <f>IF(AND(ISNUMBER(G27),ISNUMBER(H27)),H27-G27,"")</f>
-        <v/>
-      </c>
-      <c r="J27" s="8" t="n"/>
+      <c r="I27" s="8" t="n"/>
+      <c r="J27" s="8">
+        <f>IF(AND(ISNUMBER(H27),ISNUMBER(I27)),I27-H27,"")</f>
+        <v/>
+      </c>
+      <c r="K27" s="8" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="8" t="n"/>
       <c r="B28" s="8" t="n"/>
-      <c r="C28" s="8" t="n"/>
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="8" t="n"/>
       <c r="F28" s="8" t="n"/>
       <c r="G28" s="8" t="n"/>
       <c r="H28" s="8" t="n"/>
-      <c r="I28" s="8">
-        <f>IF(AND(ISNUMBER(G28),ISNUMBER(H28)),H28-G28,"")</f>
-        <v/>
-      </c>
-      <c r="J28" s="8" t="n"/>
+      <c r="I28" s="8" t="n"/>
+      <c r="J28" s="8">
+        <f>IF(AND(ISNUMBER(H28),ISNUMBER(I28)),I28-H28,"")</f>
+        <v/>
+      </c>
+      <c r="K28" s="8" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="8" t="n"/>
       <c r="B29" s="8" t="n"/>
-      <c r="C29" s="8" t="n"/>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="8" t="n"/>
       <c r="F29" s="8" t="n"/>
       <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
-      <c r="I29" s="8">
-        <f>IF(AND(ISNUMBER(G29),ISNUMBER(H29)),H29-G29,"")</f>
-        <v/>
-      </c>
-      <c r="J29" s="8" t="n"/>
+      <c r="I29" s="8" t="n"/>
+      <c r="J29" s="8">
+        <f>IF(AND(ISNUMBER(H29),ISNUMBER(I29)),I29-H29,"")</f>
+        <v/>
+      </c>
+      <c r="K29" s="8" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="8" t="n"/>
       <c r="B30" s="8" t="n"/>
-      <c r="C30" s="8" t="n"/>
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="8" t="n"/>
       <c r="F30" s="8" t="n"/>
       <c r="G30" s="8" t="n"/>
       <c r="H30" s="8" t="n"/>
-      <c r="I30" s="8">
-        <f>IF(AND(ISNUMBER(G30),ISNUMBER(H30)),H30-G30,"")</f>
-        <v/>
-      </c>
-      <c r="J30" s="8" t="n"/>
+      <c r="I30" s="8" t="n"/>
+      <c r="J30" s="8">
+        <f>IF(AND(ISNUMBER(H30),ISNUMBER(I30)),I30-H30,"")</f>
+        <v/>
+      </c>
+      <c r="K30" s="8" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="8" t="n"/>
       <c r="B31" s="8" t="n"/>
-      <c r="C31" s="8" t="n"/>
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="8" t="n"/>
       <c r="F31" s="8" t="n"/>
       <c r="G31" s="8" t="n"/>
       <c r="H31" s="8" t="n"/>
-      <c r="I31" s="8">
-        <f>IF(AND(ISNUMBER(G31),ISNUMBER(H31)),H31-G31,"")</f>
-        <v/>
-      </c>
-      <c r="J31" s="8" t="n"/>
+      <c r="I31" s="8" t="n"/>
+      <c r="J31" s="8">
+        <f>IF(AND(ISNUMBER(H31),ISNUMBER(I31)),I31-H31,"")</f>
+        <v/>
+      </c>
+      <c r="K31" s="8" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="8" t="n"/>
       <c r="B32" s="8" t="n"/>
-      <c r="C32" s="8" t="n"/>
       <c r="D32" s="8" t="n"/>
       <c r="E32" s="8" t="n"/>
       <c r="F32" s="8" t="n"/>
       <c r="G32" s="8" t="n"/>
       <c r="H32" s="8" t="n"/>
-      <c r="I32" s="8">
-        <f>IF(AND(ISNUMBER(G32),ISNUMBER(H32)),H32-G32,"")</f>
-        <v/>
-      </c>
-      <c r="J32" s="8" t="n"/>
+      <c r="I32" s="8" t="n"/>
+      <c r="J32" s="8">
+        <f>IF(AND(ISNUMBER(H32),ISNUMBER(I32)),I32-H32,"")</f>
+        <v/>
+      </c>
+      <c r="K32" s="8" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="8" t="n"/>
       <c r="B33" s="8" t="n"/>
-      <c r="C33" s="8" t="n"/>
       <c r="D33" s="8" t="n"/>
       <c r="E33" s="8" t="n"/>
       <c r="F33" s="8" t="n"/>
       <c r="G33" s="8" t="n"/>
       <c r="H33" s="8" t="n"/>
-      <c r="I33" s="8">
-        <f>IF(AND(ISNUMBER(G33),ISNUMBER(H33)),H33-G33,"")</f>
-        <v/>
-      </c>
-      <c r="J33" s="8" t="n"/>
+      <c r="I33" s="8" t="n"/>
+      <c r="J33" s="8">
+        <f>IF(AND(ISNUMBER(H33),ISNUMBER(I33)),I33-H33,"")</f>
+        <v/>
+      </c>
+      <c r="K33" s="8" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="8" t="n"/>
       <c r="B34" s="8" t="n"/>
-      <c r="C34" s="8" t="n"/>
       <c r="D34" s="8" t="n"/>
       <c r="E34" s="8" t="n"/>
       <c r="F34" s="8" t="n"/>
       <c r="G34" s="8" t="n"/>
       <c r="H34" s="8" t="n"/>
-      <c r="I34" s="8">
-        <f>IF(AND(ISNUMBER(G34),ISNUMBER(H34)),H34-G34,"")</f>
-        <v/>
-      </c>
-      <c r="J34" s="8" t="n"/>
+      <c r="I34" s="8" t="n"/>
+      <c r="J34" s="8">
+        <f>IF(AND(ISNUMBER(H34),ISNUMBER(I34)),I34-H34,"")</f>
+        <v/>
+      </c>
+      <c r="K34" s="8" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="8" t="n"/>
       <c r="B35" s="8" t="n"/>
-      <c r="C35" s="8" t="n"/>
       <c r="D35" s="8" t="n"/>
       <c r="E35" s="8" t="n"/>
       <c r="F35" s="8" t="n"/>
       <c r="G35" s="8" t="n"/>
       <c r="H35" s="8" t="n"/>
-      <c r="I35" s="8">
-        <f>IF(AND(ISNUMBER(G35),ISNUMBER(H35)),H35-G35,"")</f>
-        <v/>
-      </c>
-      <c r="J35" s="8" t="n"/>
+      <c r="I35" s="8" t="n"/>
+      <c r="J35" s="8">
+        <f>IF(AND(ISNUMBER(H35),ISNUMBER(I35)),I35-H35,"")</f>
+        <v/>
+      </c>
+      <c r="K35" s="8" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="8" t="n"/>
       <c r="B36" s="8" t="n"/>
-      <c r="C36" s="8" t="n"/>
       <c r="D36" s="8" t="n"/>
       <c r="E36" s="8" t="n"/>
       <c r="F36" s="8" t="n"/>
       <c r="G36" s="8" t="n"/>
       <c r="H36" s="8" t="n"/>
-      <c r="I36" s="8">
-        <f>IF(AND(ISNUMBER(G36),ISNUMBER(H36)),H36-G36,"")</f>
-        <v/>
-      </c>
-      <c r="J36" s="8" t="n"/>
+      <c r="I36" s="8" t="n"/>
+      <c r="J36" s="8">
+        <f>IF(AND(ISNUMBER(H36),ISNUMBER(I36)),I36-H36,"")</f>
+        <v/>
+      </c>
+      <c r="K36" s="8" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="8" t="n"/>
       <c r="B37" s="8" t="n"/>
-      <c r="C37" s="8" t="n"/>
       <c r="D37" s="8" t="n"/>
       <c r="E37" s="8" t="n"/>
       <c r="F37" s="8" t="n"/>
       <c r="G37" s="8" t="n"/>
       <c r="H37" s="8" t="n"/>
-      <c r="I37" s="8">
-        <f>IF(AND(ISNUMBER(G37),ISNUMBER(H37)),H37-G37,"")</f>
-        <v/>
-      </c>
-      <c r="J37" s="8" t="n"/>
+      <c r="I37" s="8" t="n"/>
+      <c r="J37" s="8">
+        <f>IF(AND(ISNUMBER(H37),ISNUMBER(I37)),I37-H37,"")</f>
+        <v/>
+      </c>
+      <c r="K37" s="8" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="8" t="n"/>
       <c r="B38" s="8" t="n"/>
-      <c r="C38" s="8" t="n"/>
       <c r="D38" s="8" t="n"/>
       <c r="E38" s="8" t="n"/>
       <c r="F38" s="8" t="n"/>
       <c r="G38" s="8" t="n"/>
       <c r="H38" s="8" t="n"/>
-      <c r="I38" s="8">
-        <f>IF(AND(ISNUMBER(G38),ISNUMBER(H38)),H38-G38,"")</f>
-        <v/>
-      </c>
-      <c r="J38" s="8" t="n"/>
+      <c r="I38" s="8" t="n"/>
+      <c r="J38" s="8">
+        <f>IF(AND(ISNUMBER(H38),ISNUMBER(I38)),I38-H38,"")</f>
+        <v/>
+      </c>
+      <c r="K38" s="8" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="8" t="n"/>
       <c r="B39" s="8" t="n"/>
-      <c r="C39" s="8" t="n"/>
       <c r="D39" s="8" t="n"/>
       <c r="E39" s="8" t="n"/>
       <c r="F39" s="8" t="n"/>
       <c r="G39" s="8" t="n"/>
       <c r="H39" s="8" t="n"/>
-      <c r="I39" s="8">
-        <f>IF(AND(ISNUMBER(G39),ISNUMBER(H39)),H39-G39,"")</f>
-        <v/>
-      </c>
-      <c r="J39" s="8" t="n"/>
+      <c r="I39" s="8" t="n"/>
+      <c r="J39" s="8">
+        <f>IF(AND(ISNUMBER(H39),ISNUMBER(I39)),I39-H39,"")</f>
+        <v/>
+      </c>
+      <c r="K39" s="8" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="8" t="n"/>
       <c r="B40" s="8" t="n"/>
-      <c r="C40" s="8" t="n"/>
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="8" t="n"/>
       <c r="F40" s="8" t="n"/>
       <c r="G40" s="8" t="n"/>
       <c r="H40" s="8" t="n"/>
-      <c r="I40" s="8">
-        <f>IF(AND(ISNUMBER(G40),ISNUMBER(H40)),H40-G40,"")</f>
-        <v/>
-      </c>
-      <c r="J40" s="8" t="n"/>
+      <c r="I40" s="8" t="n"/>
+      <c r="J40" s="8">
+        <f>IF(AND(ISNUMBER(H40),ISNUMBER(I40)),I40-H40,"")</f>
+        <v/>
+      </c>
+      <c r="K40" s="8" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="8" t="n"/>
       <c r="B41" s="8" t="n"/>
-      <c r="C41" s="8" t="n"/>
       <c r="D41" s="8" t="n"/>
       <c r="E41" s="8" t="n"/>
       <c r="F41" s="8" t="n"/>
       <c r="G41" s="8" t="n"/>
       <c r="H41" s="8" t="n"/>
-      <c r="I41" s="8">
-        <f>IF(AND(ISNUMBER(G41),ISNUMBER(H41)),H41-G41,"")</f>
-        <v/>
-      </c>
-      <c r="J41" s="8" t="n"/>
+      <c r="I41" s="8" t="n"/>
+      <c r="J41" s="8">
+        <f>IF(AND(ISNUMBER(H41),ISNUMBER(I41)),I41-H41,"")</f>
+        <v/>
+      </c>
+      <c r="K41" s="8" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="8" t="n"/>
       <c r="B42" s="8" t="n"/>
-      <c r="C42" s="8" t="n"/>
       <c r="D42" s="8" t="n"/>
       <c r="E42" s="8" t="n"/>
       <c r="F42" s="8" t="n"/>
       <c r="G42" s="8" t="n"/>
       <c r="H42" s="8" t="n"/>
-      <c r="I42" s="8">
-        <f>IF(AND(ISNUMBER(G42),ISNUMBER(H42)),H42-G42,"")</f>
-        <v/>
-      </c>
-      <c r="J42" s="8" t="n"/>
+      <c r="I42" s="8" t="n"/>
+      <c r="J42" s="8">
+        <f>IF(AND(ISNUMBER(H42),ISNUMBER(I42)),I42-H42,"")</f>
+        <v/>
+      </c>
+      <c r="K42" s="8" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="8" t="n"/>
       <c r="B43" s="8" t="n"/>
-      <c r="C43" s="8" t="n"/>
       <c r="D43" s="8" t="n"/>
       <c r="E43" s="8" t="n"/>
       <c r="F43" s="8" t="n"/>
       <c r="G43" s="8" t="n"/>
       <c r="H43" s="8" t="n"/>
-      <c r="I43" s="8">
-        <f>IF(AND(ISNUMBER(G43),ISNUMBER(H43)),H43-G43,"")</f>
-        <v/>
-      </c>
-      <c r="J43" s="8" t="n"/>
+      <c r="I43" s="8" t="n"/>
+      <c r="J43" s="8">
+        <f>IF(AND(ISNUMBER(H43),ISNUMBER(I43)),I43-H43,"")</f>
+        <v/>
+      </c>
+      <c r="K43" s="8" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="8" t="n"/>
       <c r="B44" s="8" t="n"/>
-      <c r="C44" s="8" t="n"/>
       <c r="D44" s="8" t="n"/>
       <c r="E44" s="8" t="n"/>
       <c r="F44" s="8" t="n"/>
       <c r="G44" s="8" t="n"/>
       <c r="H44" s="8" t="n"/>
-      <c r="I44" s="8">
-        <f>IF(AND(ISNUMBER(G44),ISNUMBER(H44)),H44-G44,"")</f>
-        <v/>
-      </c>
-      <c r="J44" s="8" t="n"/>
+      <c r="I44" s="8" t="n"/>
+      <c r="J44" s="8">
+        <f>IF(AND(ISNUMBER(H44),ISNUMBER(I44)),I44-H44,"")</f>
+        <v/>
+      </c>
+      <c r="K44" s="8" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="8" t="n"/>
       <c r="B45" s="8" t="n"/>
-      <c r="C45" s="8" t="n"/>
       <c r="D45" s="8" t="n"/>
       <c r="E45" s="8" t="n"/>
       <c r="F45" s="8" t="n"/>
       <c r="G45" s="8" t="n"/>
       <c r="H45" s="8" t="n"/>
-      <c r="I45" s="8">
-        <f>IF(AND(ISNUMBER(G45),ISNUMBER(H45)),H45-G45,"")</f>
-        <v/>
-      </c>
-      <c r="J45" s="8" t="n"/>
+      <c r="I45" s="8" t="n"/>
+      <c r="J45" s="8">
+        <f>IF(AND(ISNUMBER(H45),ISNUMBER(I45)),I45-H45,"")</f>
+        <v/>
+      </c>
+      <c r="K45" s="8" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="8" t="n"/>
       <c r="B46" s="8" t="n"/>
-      <c r="C46" s="8" t="n"/>
       <c r="D46" s="8" t="n"/>
       <c r="E46" s="8" t="n"/>
       <c r="F46" s="8" t="n"/>
       <c r="G46" s="8" t="n"/>
       <c r="H46" s="8" t="n"/>
-      <c r="I46" s="8">
-        <f>IF(AND(ISNUMBER(G46),ISNUMBER(H46)),H46-G46,"")</f>
-        <v/>
-      </c>
-      <c r="J46" s="8" t="n"/>
+      <c r="I46" s="8" t="n"/>
+      <c r="J46" s="8">
+        <f>IF(AND(ISNUMBER(H46),ISNUMBER(I46)),I46-H46,"")</f>
+        <v/>
+      </c>
+      <c r="K46" s="8" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="8" t="n"/>
       <c r="B47" s="8" t="n"/>
-      <c r="C47" s="8" t="n"/>
       <c r="D47" s="8" t="n"/>
       <c r="E47" s="8" t="n"/>
       <c r="F47" s="8" t="n"/>
       <c r="G47" s="8" t="n"/>
       <c r="H47" s="8" t="n"/>
-      <c r="I47" s="8">
-        <f>IF(AND(ISNUMBER(G47),ISNUMBER(H47)),H47-G47,"")</f>
-        <v/>
-      </c>
-      <c r="J47" s="8" t="n"/>
+      <c r="I47" s="8" t="n"/>
+      <c r="J47" s="8">
+        <f>IF(AND(ISNUMBER(H47),ISNUMBER(I47)),I47-H47,"")</f>
+        <v/>
+      </c>
+      <c r="K47" s="8" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="8" t="n"/>
       <c r="B48" s="8" t="n"/>
-      <c r="C48" s="8" t="n"/>
       <c r="D48" s="8" t="n"/>
       <c r="E48" s="8" t="n"/>
       <c r="F48" s="8" t="n"/>
       <c r="G48" s="8" t="n"/>
       <c r="H48" s="8" t="n"/>
-      <c r="I48" s="8">
-        <f>IF(AND(ISNUMBER(G48),ISNUMBER(H48)),H48-G48,"")</f>
-        <v/>
-      </c>
-      <c r="J48" s="8" t="n"/>
+      <c r="I48" s="8" t="n"/>
+      <c r="J48" s="8">
+        <f>IF(AND(ISNUMBER(H48),ISNUMBER(I48)),I48-H48,"")</f>
+        <v/>
+      </c>
+      <c r="K48" s="8" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="8" t="n"/>
       <c r="B49" s="8" t="n"/>
-      <c r="C49" s="8" t="n"/>
       <c r="D49" s="8" t="n"/>
       <c r="E49" s="8" t="n"/>
       <c r="F49" s="8" t="n"/>
       <c r="G49" s="8" t="n"/>
       <c r="H49" s="8" t="n"/>
-      <c r="I49" s="8">
-        <f>IF(AND(ISNUMBER(G49),ISNUMBER(H49)),H49-G49,"")</f>
-        <v/>
-      </c>
-      <c r="J49" s="8" t="n"/>
+      <c r="I49" s="8" t="n"/>
+      <c r="J49" s="8">
+        <f>IF(AND(ISNUMBER(H49),ISNUMBER(I49)),I49-H49,"")</f>
+        <v/>
+      </c>
+      <c r="K49" s="8" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="8" t="n"/>
       <c r="B50" s="8" t="n"/>
-      <c r="C50" s="8" t="n"/>
       <c r="D50" s="8" t="n"/>
       <c r="E50" s="8" t="n"/>
       <c r="F50" s="8" t="n"/>
       <c r="G50" s="8" t="n"/>
       <c r="H50" s="8" t="n"/>
-      <c r="I50" s="8">
-        <f>IF(AND(ISNUMBER(G50),ISNUMBER(H50)),H50-G50,"")</f>
-        <v/>
-      </c>
-      <c r="J50" s="8" t="n"/>
+      <c r="I50" s="8" t="n"/>
+      <c r="J50" s="8">
+        <f>IF(AND(ISNUMBER(H50),ISNUMBER(I50)),I50-H50,"")</f>
+        <v/>
+      </c>
+      <c r="K50" s="8" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="8" t="n"/>
       <c r="B51" s="8" t="n"/>
-      <c r="C51" s="8" t="n"/>
       <c r="D51" s="8" t="n"/>
       <c r="E51" s="8" t="n"/>
       <c r="F51" s="8" t="n"/>
       <c r="G51" s="8" t="n"/>
       <c r="H51" s="8" t="n"/>
-      <c r="I51" s="8">
-        <f>IF(AND(ISNUMBER(G51),ISNUMBER(H51)),H51-G51,"")</f>
-        <v/>
-      </c>
-      <c r="J51" s="8" t="n"/>
+      <c r="I51" s="8" t="n"/>
+      <c r="J51" s="8">
+        <f>IF(AND(ISNUMBER(H51),ISNUMBER(I51)),I51-H51,"")</f>
+        <v/>
+      </c>
+      <c r="K51" s="8" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="8" t="n"/>
       <c r="B52" s="8" t="n"/>
-      <c r="C52" s="8" t="n"/>
       <c r="D52" s="8" t="n"/>
       <c r="E52" s="8" t="n"/>
       <c r="F52" s="8" t="n"/>
       <c r="G52" s="8" t="n"/>
       <c r="H52" s="8" t="n"/>
-      <c r="I52" s="8">
-        <f>IF(AND(ISNUMBER(G52),ISNUMBER(H52)),H52-G52,"")</f>
-        <v/>
-      </c>
-      <c r="J52" s="8" t="n"/>
+      <c r="I52" s="8" t="n"/>
+      <c r="J52" s="8">
+        <f>IF(AND(ISNUMBER(H52),ISNUMBER(I52)),I52-H52,"")</f>
+        <v/>
+      </c>
+      <c r="K52" s="8" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="8" t="n"/>
       <c r="B53" s="8" t="n"/>
-      <c r="C53" s="8" t="n"/>
       <c r="D53" s="8" t="n"/>
       <c r="E53" s="8" t="n"/>
       <c r="F53" s="8" t="n"/>
       <c r="G53" s="8" t="n"/>
       <c r="H53" s="8" t="n"/>
-      <c r="I53" s="8">
-        <f>IF(AND(ISNUMBER(G53),ISNUMBER(H53)),H53-G53,"")</f>
-        <v/>
-      </c>
-      <c r="J53" s="8" t="n"/>
+      <c r="I53" s="8" t="n"/>
+      <c r="J53" s="8">
+        <f>IF(AND(ISNUMBER(H53),ISNUMBER(I53)),I53-H53,"")</f>
+        <v/>
+      </c>
+      <c r="K53" s="8" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="8" t="n"/>
       <c r="B54" s="8" t="n"/>
-      <c r="C54" s="8" t="n"/>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="8" t="n"/>
       <c r="F54" s="8" t="n"/>
       <c r="G54" s="8" t="n"/>
       <c r="H54" s="8" t="n"/>
-      <c r="I54" s="8">
-        <f>IF(AND(ISNUMBER(G54),ISNUMBER(H54)),H54-G54,"")</f>
-        <v/>
-      </c>
-      <c r="J54" s="8" t="n"/>
+      <c r="I54" s="8" t="n"/>
+      <c r="J54" s="8">
+        <f>IF(AND(ISNUMBER(H54),ISNUMBER(I54)),I54-H54,"")</f>
+        <v/>
+      </c>
+      <c r="K54" s="8" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="8" t="n"/>
       <c r="B55" s="8" t="n"/>
-      <c r="C55" s="8" t="n"/>
       <c r="D55" s="8" t="n"/>
       <c r="E55" s="8" t="n"/>
       <c r="F55" s="8" t="n"/>
       <c r="G55" s="8" t="n"/>
       <c r="H55" s="8" t="n"/>
-      <c r="I55" s="8">
-        <f>IF(AND(ISNUMBER(G55),ISNUMBER(H55)),H55-G55,"")</f>
-        <v/>
-      </c>
-      <c r="J55" s="8" t="n"/>
+      <c r="I55" s="8" t="n"/>
+      <c r="J55" s="8">
+        <f>IF(AND(ISNUMBER(H55),ISNUMBER(I55)),I55-H55,"")</f>
+        <v/>
+      </c>
+      <c r="K55" s="8" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="8" t="n"/>
       <c r="B56" s="8" t="n"/>
-      <c r="C56" s="8" t="n"/>
       <c r="D56" s="8" t="n"/>
       <c r="E56" s="8" t="n"/>
       <c r="F56" s="8" t="n"/>
       <c r="G56" s="8" t="n"/>
       <c r="H56" s="8" t="n"/>
-      <c r="I56" s="8">
-        <f>IF(AND(ISNUMBER(G56),ISNUMBER(H56)),H56-G56,"")</f>
-        <v/>
-      </c>
-      <c r="J56" s="8" t="n"/>
+      <c r="I56" s="8" t="n"/>
+      <c r="J56" s="8">
+        <f>IF(AND(ISNUMBER(H56),ISNUMBER(I56)),I56-H56,"")</f>
+        <v/>
+      </c>
+      <c r="K56" s="8" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="8" t="n"/>
       <c r="B57" s="8" t="n"/>
-      <c r="C57" s="8" t="n"/>
       <c r="D57" s="8" t="n"/>
       <c r="E57" s="8" t="n"/>
       <c r="F57" s="8" t="n"/>
       <c r="G57" s="8" t="n"/>
       <c r="H57" s="8" t="n"/>
-      <c r="I57" s="8">
-        <f>IF(AND(ISNUMBER(G57),ISNUMBER(H57)),H57-G57,"")</f>
-        <v/>
-      </c>
-      <c r="J57" s="8" t="n"/>
+      <c r="I57" s="8" t="n"/>
+      <c r="J57" s="8">
+        <f>IF(AND(ISNUMBER(H57),ISNUMBER(I57)),I57-H57,"")</f>
+        <v/>
+      </c>
+      <c r="K57" s="8" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="8" t="n"/>
       <c r="B58" s="8" t="n"/>
-      <c r="C58" s="8" t="n"/>
       <c r="D58" s="8" t="n"/>
       <c r="E58" s="8" t="n"/>
       <c r="F58" s="8" t="n"/>
       <c r="G58" s="8" t="n"/>
       <c r="H58" s="8" t="n"/>
-      <c r="I58" s="8">
-        <f>IF(AND(ISNUMBER(G58),ISNUMBER(H58)),H58-G58,"")</f>
-        <v/>
-      </c>
-      <c r="J58" s="8" t="n"/>
+      <c r="I58" s="8" t="n"/>
+      <c r="J58" s="8">
+        <f>IF(AND(ISNUMBER(H58),ISNUMBER(I58)),I58-H58,"")</f>
+        <v/>
+      </c>
+      <c r="K58" s="8" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="8" t="n"/>
       <c r="B59" s="8" t="n"/>
-      <c r="C59" s="8" t="n"/>
       <c r="D59" s="8" t="n"/>
       <c r="E59" s="8" t="n"/>
       <c r="F59" s="8" t="n"/>
       <c r="G59" s="8" t="n"/>
       <c r="H59" s="8" t="n"/>
-      <c r="I59" s="8">
-        <f>IF(AND(ISNUMBER(G59),ISNUMBER(H59)),H59-G59,"")</f>
-        <v/>
-      </c>
-      <c r="J59" s="8" t="n"/>
+      <c r="I59" s="8" t="n"/>
+      <c r="J59" s="8">
+        <f>IF(AND(ISNUMBER(H59),ISNUMBER(I59)),I59-H59,"")</f>
+        <v/>
+      </c>
+      <c r="K59" s="8" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="8" t="n"/>
       <c r="B60" s="8" t="n"/>
-      <c r="C60" s="8" t="n"/>
       <c r="D60" s="8" t="n"/>
       <c r="E60" s="8" t="n"/>
       <c r="F60" s="8" t="n"/>
       <c r="G60" s="8" t="n"/>
       <c r="H60" s="8" t="n"/>
-      <c r="I60" s="8">
-        <f>IF(AND(ISNUMBER(G60),ISNUMBER(H60)),H60-G60,"")</f>
-        <v/>
-      </c>
-      <c r="J60" s="8" t="n"/>
+      <c r="I60" s="8" t="n"/>
+      <c r="J60" s="8">
+        <f>IF(AND(ISNUMBER(H60),ISNUMBER(I60)),I60-H60,"")</f>
+        <v/>
+      </c>
+      <c r="K60" s="8" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="8" t="n"/>
       <c r="B61" s="8" t="n"/>
-      <c r="C61" s="8" t="n"/>
       <c r="D61" s="8" t="n"/>
       <c r="E61" s="8" t="n"/>
       <c r="F61" s="8" t="n"/>
       <c r="G61" s="8" t="n"/>
       <c r="H61" s="8" t="n"/>
-      <c r="I61" s="8">
-        <f>IF(AND(ISNUMBER(G61),ISNUMBER(H61)),H61-G61,"")</f>
-        <v/>
-      </c>
-      <c r="J61" s="8" t="n"/>
+      <c r="I61" s="8" t="n"/>
+      <c r="J61" s="8">
+        <f>IF(AND(ISNUMBER(H61),ISNUMBER(I61)),I61-H61,"")</f>
+        <v/>
+      </c>
+      <c r="K61" s="8" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="8" t="n"/>
       <c r="B62" s="8" t="n"/>
-      <c r="C62" s="8" t="n"/>
       <c r="D62" s="8" t="n"/>
       <c r="E62" s="8" t="n"/>
       <c r="F62" s="8" t="n"/>
       <c r="G62" s="8" t="n"/>
       <c r="H62" s="8" t="n"/>
-      <c r="I62" s="8">
-        <f>IF(AND(ISNUMBER(G62),ISNUMBER(H62)),H62-G62,"")</f>
-        <v/>
-      </c>
-      <c r="J62" s="8" t="n"/>
+      <c r="I62" s="8" t="n"/>
+      <c r="J62" s="8">
+        <f>IF(AND(ISNUMBER(H62),ISNUMBER(I62)),I62-H62,"")</f>
+        <v/>
+      </c>
+      <c r="K62" s="8" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="8" t="n"/>
       <c r="B63" s="8" t="n"/>
-      <c r="C63" s="8" t="n"/>
       <c r="D63" s="8" t="n"/>
       <c r="E63" s="8" t="n"/>
       <c r="F63" s="8" t="n"/>
       <c r="G63" s="8" t="n"/>
       <c r="H63" s="8" t="n"/>
-      <c r="I63" s="8">
-        <f>IF(AND(ISNUMBER(G63),ISNUMBER(H63)),H63-G63,"")</f>
-        <v/>
-      </c>
-      <c r="J63" s="8" t="n"/>
+      <c r="I63" s="8" t="n"/>
+      <c r="J63" s="8">
+        <f>IF(AND(ISNUMBER(H63),ISNUMBER(I63)),I63-H63,"")</f>
+        <v/>
+      </c>
+      <c r="K63" s="8" t="n"/>
     </row>
   </sheetData>
-  <dataValidations count="1">
+  <dataValidations count="3">
     <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Low,Med,High"</formula1>
+    </dataValidation>
+    <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Top level,Concepts,API,SDKs,Guides,Operations,Reference,External,Other"</formula1>
+    </dataValidation>
+    <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Med,High"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Drop numeric-score framing — tool reports pass/warning per signal only. Reframe README + CONTRIBUTING + tracker + issue footers around 'did the tool detect your fix? give honest feedback'
</commit_message>
<xml_diff>
--- a/pattern-tracker.xlsx
+++ b/pattern-tracker.xlsx
@@ -18,7 +18,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="12">
+  <fonts count="13">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -82,6 +82,12 @@
     <font>
       <b val="1"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <i val="1"/>
+      <color rgb="0028251D"/>
+      <sz val="11"/>
+    </font>
   </fonts>
   <fills count="3">
     <fill>
@@ -122,7 +128,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="13">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
@@ -156,6 +162,12 @@
     </xf>
     <xf numFmtId="0" fontId="10" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="11" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -559,7 +571,11 @@
       </c>
     </row>
     <row r="6">
-      <c r="A6" s="3" t="inlineStr"/>
+      <c r="A6" s="13" t="inlineStr">
+        <is>
+          <t>Note: the audit tool currently reports pass / warning / not-verified per signal — there is no numeric score. Honest feedback about the tool itself (including "the tool missed my fix") is what we want to capture.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
@@ -613,26 +629,30 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>7. Score Before / After — from the audit tool</t>
+          <t>7. Tool detected fix? — did the audit tool pick up your change? (Yes / Partial / No)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="3" t="inlineStr">
         <is>
-          <t>8. Score Delta — auto-calculated</t>
+          <t>8. Signal that moved — short note: which signal flipped, e.g. "llms.txt went from ✗ to ✓"</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>9. Notes — anything else worth remembering</t>
+          <t>9. Honest feedback on tool — open-ended. If the tool missed your fix, say so. If it caught something interesting, say that too.</t>
         </is>
       </c>
     </row>
     <row r="17">
-      <c r="A17" s="3" t="inlineStr"/>
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>10. Notes — anything else worth remembering</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
@@ -748,7 +768,6 @@
         </is>
       </c>
     </row>
-    <row r="36"/>
     <row r="37">
       <c r="A37" s="11" t="inlineStr">
         <is>
@@ -770,7 +789,6 @@
         </is>
       </c>
     </row>
-    <row r="40"/>
     <row r="41">
       <c r="A41" s="11" t="inlineStr">
         <is>
@@ -792,7 +810,6 @@
         </is>
       </c>
     </row>
-    <row r="44"/>
     <row r="45">
       <c r="A45" s="11" t="inlineStr">
         <is>
@@ -870,9 +887,9 @@
     <col width="40" customWidth="1" min="5" max="5"/>
     <col width="10" customWidth="1" min="6" max="6"/>
     <col width="38" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="14" customWidth="1" min="9" max="9"/>
-    <col width="12" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="50" customWidth="1" min="9" max="9"/>
+    <col width="50" customWidth="1" min="10" max="10"/>
     <col width="35" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
@@ -914,17 +931,17 @@
       </c>
       <c r="H1" s="6" t="inlineStr">
         <is>
-          <t>Score Before</t>
+          <t>Tool detected fix?</t>
         </is>
       </c>
       <c r="I1" s="6" t="inlineStr">
         <is>
-          <t>Score After</t>
+          <t>Signal that moved</t>
         </is>
       </c>
       <c r="J1" s="6" t="inlineStr">
         <is>
-          <t>Score Delta</t>
+          <t>Honest feedback on tool</t>
         </is>
       </c>
       <c r="K1" s="6" t="inlineStr">
@@ -967,15 +984,20 @@
           <t>Split into H2 per endpoint with request/response example each</t>
         </is>
       </c>
-      <c r="H2" s="7" t="n">
-        <v>42</v>
-      </c>
-      <c r="I2" s="7" t="n">
-        <v>71</v>
-      </c>
-      <c r="J2" s="7">
-        <f>I2-H2</f>
-        <v/>
+      <c r="H2" s="14" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="I2" s="14" t="inlineStr">
+        <is>
+          <t>Content Quality: structure heading flipped from ⚠ to ✓; endpoints now show as own sections</t>
+        </is>
+      </c>
+      <c r="J2" s="14" t="inlineStr">
+        <is>
+          <t>Tool caught the structural change immediately. Did NOT comment on whether request/response examples were complete — would be useful.</t>
+        </is>
       </c>
       <c r="K2" s="7" t="inlineStr">
         <is>
@@ -1019,15 +1041,20 @@
           <t>Added language tags to 12 code samples</t>
         </is>
       </c>
-      <c r="H3" s="7" t="n">
-        <v>58</v>
-      </c>
-      <c r="I3" s="7" t="n">
-        <v>73</v>
-      </c>
-      <c r="J3" s="7">
-        <f>I3-H3</f>
-        <v/>
+      <c r="H3" s="14" t="inlineStr">
+        <is>
+          <t>Partial</t>
+        </is>
+      </c>
+      <c r="I3" s="14" t="inlineStr">
+        <is>
+          <t>Code blocks now show as language-tagged in the report; site-level Discoverability still warning (no llms.txt yet)</t>
+        </is>
+      </c>
+      <c r="J3" s="14" t="inlineStr">
+        <is>
+          <t>Tool flagged language tags fine. Missed that one block was tagged `js` but the site uses `javascript` elsewhere — inconsistency the tool didn't catch.</t>
+        </is>
       </c>
       <c r="K3" s="7" t="inlineStr">
         <is>
@@ -1044,10 +1071,7 @@
       <c r="G4" s="8" t="n"/>
       <c r="H4" s="8" t="n"/>
       <c r="I4" s="8" t="n"/>
-      <c r="J4" s="8">
-        <f>IF(AND(ISNUMBER(H4),ISNUMBER(I4)),I4-H4,"")</f>
-        <v/>
-      </c>
+      <c r="J4" s="8" t="n"/>
       <c r="K4" s="8" t="n"/>
     </row>
     <row r="5">
@@ -1059,10 +1083,7 @@
       <c r="G5" s="8" t="n"/>
       <c r="H5" s="8" t="n"/>
       <c r="I5" s="8" t="n"/>
-      <c r="J5" s="8">
-        <f>IF(AND(ISNUMBER(H5),ISNUMBER(I5)),I5-H5,"")</f>
-        <v/>
-      </c>
+      <c r="J5" s="8" t="n"/>
       <c r="K5" s="8" t="n"/>
     </row>
     <row r="6">
@@ -1074,10 +1095,7 @@
       <c r="G6" s="8" t="n"/>
       <c r="H6" s="8" t="n"/>
       <c r="I6" s="8" t="n"/>
-      <c r="J6" s="8">
-        <f>IF(AND(ISNUMBER(H6),ISNUMBER(I6)),I6-H6,"")</f>
-        <v/>
-      </c>
+      <c r="J6" s="8" t="n"/>
       <c r="K6" s="8" t="n"/>
     </row>
     <row r="7">
@@ -1089,10 +1107,7 @@
       <c r="G7" s="8" t="n"/>
       <c r="H7" s="8" t="n"/>
       <c r="I7" s="8" t="n"/>
-      <c r="J7" s="8">
-        <f>IF(AND(ISNUMBER(H7),ISNUMBER(I7)),I7-H7,"")</f>
-        <v/>
-      </c>
+      <c r="J7" s="8" t="n"/>
       <c r="K7" s="8" t="n"/>
     </row>
     <row r="8">
@@ -1104,10 +1119,7 @@
       <c r="G8" s="8" t="n"/>
       <c r="H8" s="8" t="n"/>
       <c r="I8" s="8" t="n"/>
-      <c r="J8" s="8">
-        <f>IF(AND(ISNUMBER(H8),ISNUMBER(I8)),I8-H8,"")</f>
-        <v/>
-      </c>
+      <c r="J8" s="8" t="n"/>
       <c r="K8" s="8" t="n"/>
     </row>
     <row r="9">
@@ -1119,10 +1131,7 @@
       <c r="G9" s="8" t="n"/>
       <c r="H9" s="8" t="n"/>
       <c r="I9" s="8" t="n"/>
-      <c r="J9" s="8">
-        <f>IF(AND(ISNUMBER(H9),ISNUMBER(I9)),I9-H9,"")</f>
-        <v/>
-      </c>
+      <c r="J9" s="8" t="n"/>
       <c r="K9" s="8" t="n"/>
     </row>
     <row r="10">
@@ -1134,10 +1143,7 @@
       <c r="G10" s="8" t="n"/>
       <c r="H10" s="8" t="n"/>
       <c r="I10" s="8" t="n"/>
-      <c r="J10" s="8">
-        <f>IF(AND(ISNUMBER(H10),ISNUMBER(I10)),I10-H10,"")</f>
-        <v/>
-      </c>
+      <c r="J10" s="8" t="n"/>
       <c r="K10" s="8" t="n"/>
     </row>
     <row r="11">
@@ -1149,10 +1155,7 @@
       <c r="G11" s="8" t="n"/>
       <c r="H11" s="8" t="n"/>
       <c r="I11" s="8" t="n"/>
-      <c r="J11" s="8">
-        <f>IF(AND(ISNUMBER(H11),ISNUMBER(I11)),I11-H11,"")</f>
-        <v/>
-      </c>
+      <c r="J11" s="8" t="n"/>
       <c r="K11" s="8" t="n"/>
     </row>
     <row r="12">
@@ -1164,10 +1167,7 @@
       <c r="G12" s="8" t="n"/>
       <c r="H12" s="8" t="n"/>
       <c r="I12" s="8" t="n"/>
-      <c r="J12" s="8">
-        <f>IF(AND(ISNUMBER(H12),ISNUMBER(I12)),I12-H12,"")</f>
-        <v/>
-      </c>
+      <c r="J12" s="8" t="n"/>
       <c r="K12" s="8" t="n"/>
     </row>
     <row r="13">
@@ -1179,10 +1179,7 @@
       <c r="G13" s="8" t="n"/>
       <c r="H13" s="8" t="n"/>
       <c r="I13" s="8" t="n"/>
-      <c r="J13" s="8">
-        <f>IF(AND(ISNUMBER(H13),ISNUMBER(I13)),I13-H13,"")</f>
-        <v/>
-      </c>
+      <c r="J13" s="8" t="n"/>
       <c r="K13" s="8" t="n"/>
     </row>
     <row r="14">
@@ -1194,10 +1191,7 @@
       <c r="G14" s="8" t="n"/>
       <c r="H14" s="8" t="n"/>
       <c r="I14" s="8" t="n"/>
-      <c r="J14" s="8">
-        <f>IF(AND(ISNUMBER(H14),ISNUMBER(I14)),I14-H14,"")</f>
-        <v/>
-      </c>
+      <c r="J14" s="8" t="n"/>
       <c r="K14" s="8" t="n"/>
     </row>
     <row r="15">
@@ -1209,10 +1203,7 @@
       <c r="G15" s="8" t="n"/>
       <c r="H15" s="8" t="n"/>
       <c r="I15" s="8" t="n"/>
-      <c r="J15" s="8">
-        <f>IF(AND(ISNUMBER(H15),ISNUMBER(I15)),I15-H15,"")</f>
-        <v/>
-      </c>
+      <c r="J15" s="8" t="n"/>
       <c r="K15" s="8" t="n"/>
     </row>
     <row r="16">
@@ -1224,10 +1215,7 @@
       <c r="G16" s="8" t="n"/>
       <c r="H16" s="8" t="n"/>
       <c r="I16" s="8" t="n"/>
-      <c r="J16" s="8">
-        <f>IF(AND(ISNUMBER(H16),ISNUMBER(I16)),I16-H16,"")</f>
-        <v/>
-      </c>
+      <c r="J16" s="8" t="n"/>
       <c r="K16" s="8" t="n"/>
     </row>
     <row r="17">
@@ -1239,10 +1227,7 @@
       <c r="G17" s="8" t="n"/>
       <c r="H17" s="8" t="n"/>
       <c r="I17" s="8" t="n"/>
-      <c r="J17" s="8">
-        <f>IF(AND(ISNUMBER(H17),ISNUMBER(I17)),I17-H17,"")</f>
-        <v/>
-      </c>
+      <c r="J17" s="8" t="n"/>
       <c r="K17" s="8" t="n"/>
     </row>
     <row r="18">
@@ -1254,10 +1239,7 @@
       <c r="G18" s="8" t="n"/>
       <c r="H18" s="8" t="n"/>
       <c r="I18" s="8" t="n"/>
-      <c r="J18" s="8">
-        <f>IF(AND(ISNUMBER(H18),ISNUMBER(I18)),I18-H18,"")</f>
-        <v/>
-      </c>
+      <c r="J18" s="8" t="n"/>
       <c r="K18" s="8" t="n"/>
     </row>
     <row r="19">
@@ -1269,10 +1251,7 @@
       <c r="G19" s="8" t="n"/>
       <c r="H19" s="8" t="n"/>
       <c r="I19" s="8" t="n"/>
-      <c r="J19" s="8">
-        <f>IF(AND(ISNUMBER(H19),ISNUMBER(I19)),I19-H19,"")</f>
-        <v/>
-      </c>
+      <c r="J19" s="8" t="n"/>
       <c r="K19" s="8" t="n"/>
     </row>
     <row r="20">
@@ -1284,10 +1263,7 @@
       <c r="G20" s="8" t="n"/>
       <c r="H20" s="8" t="n"/>
       <c r="I20" s="8" t="n"/>
-      <c r="J20" s="8">
-        <f>IF(AND(ISNUMBER(H20),ISNUMBER(I20)),I20-H20,"")</f>
-        <v/>
-      </c>
+      <c r="J20" s="8" t="n"/>
       <c r="K20" s="8" t="n"/>
     </row>
     <row r="21">
@@ -1299,10 +1275,7 @@
       <c r="G21" s="8" t="n"/>
       <c r="H21" s="8" t="n"/>
       <c r="I21" s="8" t="n"/>
-      <c r="J21" s="8">
-        <f>IF(AND(ISNUMBER(H21),ISNUMBER(I21)),I21-H21,"")</f>
-        <v/>
-      </c>
+      <c r="J21" s="8" t="n"/>
       <c r="K21" s="8" t="n"/>
     </row>
     <row r="22">
@@ -1314,10 +1287,7 @@
       <c r="G22" s="8" t="n"/>
       <c r="H22" s="8" t="n"/>
       <c r="I22" s="8" t="n"/>
-      <c r="J22" s="8">
-        <f>IF(AND(ISNUMBER(H22),ISNUMBER(I22)),I22-H22,"")</f>
-        <v/>
-      </c>
+      <c r="J22" s="8" t="n"/>
       <c r="K22" s="8" t="n"/>
     </row>
     <row r="23">
@@ -1329,10 +1299,7 @@
       <c r="G23" s="8" t="n"/>
       <c r="H23" s="8" t="n"/>
       <c r="I23" s="8" t="n"/>
-      <c r="J23" s="8">
-        <f>IF(AND(ISNUMBER(H23),ISNUMBER(I23)),I23-H23,"")</f>
-        <v/>
-      </c>
+      <c r="J23" s="8" t="n"/>
       <c r="K23" s="8" t="n"/>
     </row>
     <row r="24">
@@ -1344,10 +1311,7 @@
       <c r="G24" s="8" t="n"/>
       <c r="H24" s="8" t="n"/>
       <c r="I24" s="8" t="n"/>
-      <c r="J24" s="8">
-        <f>IF(AND(ISNUMBER(H24),ISNUMBER(I24)),I24-H24,"")</f>
-        <v/>
-      </c>
+      <c r="J24" s="8" t="n"/>
       <c r="K24" s="8" t="n"/>
     </row>
     <row r="25">
@@ -1359,10 +1323,7 @@
       <c r="G25" s="8" t="n"/>
       <c r="H25" s="8" t="n"/>
       <c r="I25" s="8" t="n"/>
-      <c r="J25" s="8">
-        <f>IF(AND(ISNUMBER(H25),ISNUMBER(I25)),I25-H25,"")</f>
-        <v/>
-      </c>
+      <c r="J25" s="8" t="n"/>
       <c r="K25" s="8" t="n"/>
     </row>
     <row r="26">
@@ -1374,10 +1335,7 @@
       <c r="G26" s="8" t="n"/>
       <c r="H26" s="8" t="n"/>
       <c r="I26" s="8" t="n"/>
-      <c r="J26" s="8">
-        <f>IF(AND(ISNUMBER(H26),ISNUMBER(I26)),I26-H26,"")</f>
-        <v/>
-      </c>
+      <c r="J26" s="8" t="n"/>
       <c r="K26" s="8" t="n"/>
     </row>
     <row r="27">
@@ -1389,10 +1347,7 @@
       <c r="G27" s="8" t="n"/>
       <c r="H27" s="8" t="n"/>
       <c r="I27" s="8" t="n"/>
-      <c r="J27" s="8">
-        <f>IF(AND(ISNUMBER(H27),ISNUMBER(I27)),I27-H27,"")</f>
-        <v/>
-      </c>
+      <c r="J27" s="8" t="n"/>
       <c r="K27" s="8" t="n"/>
     </row>
     <row r="28">
@@ -1404,10 +1359,7 @@
       <c r="G28" s="8" t="n"/>
       <c r="H28" s="8" t="n"/>
       <c r="I28" s="8" t="n"/>
-      <c r="J28" s="8">
-        <f>IF(AND(ISNUMBER(H28),ISNUMBER(I28)),I28-H28,"")</f>
-        <v/>
-      </c>
+      <c r="J28" s="8" t="n"/>
       <c r="K28" s="8" t="n"/>
     </row>
     <row r="29">
@@ -1419,10 +1371,7 @@
       <c r="G29" s="8" t="n"/>
       <c r="H29" s="8" t="n"/>
       <c r="I29" s="8" t="n"/>
-      <c r="J29" s="8">
-        <f>IF(AND(ISNUMBER(H29),ISNUMBER(I29)),I29-H29,"")</f>
-        <v/>
-      </c>
+      <c r="J29" s="8" t="n"/>
       <c r="K29" s="8" t="n"/>
     </row>
     <row r="30">
@@ -1434,10 +1383,7 @@
       <c r="G30" s="8" t="n"/>
       <c r="H30" s="8" t="n"/>
       <c r="I30" s="8" t="n"/>
-      <c r="J30" s="8">
-        <f>IF(AND(ISNUMBER(H30),ISNUMBER(I30)),I30-H30,"")</f>
-        <v/>
-      </c>
+      <c r="J30" s="8" t="n"/>
       <c r="K30" s="8" t="n"/>
     </row>
     <row r="31">
@@ -1449,10 +1395,7 @@
       <c r="G31" s="8" t="n"/>
       <c r="H31" s="8" t="n"/>
       <c r="I31" s="8" t="n"/>
-      <c r="J31" s="8">
-        <f>IF(AND(ISNUMBER(H31),ISNUMBER(I31)),I31-H31,"")</f>
-        <v/>
-      </c>
+      <c r="J31" s="8" t="n"/>
       <c r="K31" s="8" t="n"/>
     </row>
     <row r="32">
@@ -1464,10 +1407,7 @@
       <c r="G32" s="8" t="n"/>
       <c r="H32" s="8" t="n"/>
       <c r="I32" s="8" t="n"/>
-      <c r="J32" s="8">
-        <f>IF(AND(ISNUMBER(H32),ISNUMBER(I32)),I32-H32,"")</f>
-        <v/>
-      </c>
+      <c r="J32" s="8" t="n"/>
       <c r="K32" s="8" t="n"/>
     </row>
     <row r="33">
@@ -1479,10 +1419,7 @@
       <c r="G33" s="8" t="n"/>
       <c r="H33" s="8" t="n"/>
       <c r="I33" s="8" t="n"/>
-      <c r="J33" s="8">
-        <f>IF(AND(ISNUMBER(H33),ISNUMBER(I33)),I33-H33,"")</f>
-        <v/>
-      </c>
+      <c r="J33" s="8" t="n"/>
       <c r="K33" s="8" t="n"/>
     </row>
     <row r="34">
@@ -1494,10 +1431,7 @@
       <c r="G34" s="8" t="n"/>
       <c r="H34" s="8" t="n"/>
       <c r="I34" s="8" t="n"/>
-      <c r="J34" s="8">
-        <f>IF(AND(ISNUMBER(H34),ISNUMBER(I34)),I34-H34,"")</f>
-        <v/>
-      </c>
+      <c r="J34" s="8" t="n"/>
       <c r="K34" s="8" t="n"/>
     </row>
     <row r="35">
@@ -1509,10 +1443,7 @@
       <c r="G35" s="8" t="n"/>
       <c r="H35" s="8" t="n"/>
       <c r="I35" s="8" t="n"/>
-      <c r="J35" s="8">
-        <f>IF(AND(ISNUMBER(H35),ISNUMBER(I35)),I35-H35,"")</f>
-        <v/>
-      </c>
+      <c r="J35" s="8" t="n"/>
       <c r="K35" s="8" t="n"/>
     </row>
     <row r="36">
@@ -1524,10 +1455,7 @@
       <c r="G36" s="8" t="n"/>
       <c r="H36" s="8" t="n"/>
       <c r="I36" s="8" t="n"/>
-      <c r="J36" s="8">
-        <f>IF(AND(ISNUMBER(H36),ISNUMBER(I36)),I36-H36,"")</f>
-        <v/>
-      </c>
+      <c r="J36" s="8" t="n"/>
       <c r="K36" s="8" t="n"/>
     </row>
     <row r="37">
@@ -1539,10 +1467,7 @@
       <c r="G37" s="8" t="n"/>
       <c r="H37" s="8" t="n"/>
       <c r="I37" s="8" t="n"/>
-      <c r="J37" s="8">
-        <f>IF(AND(ISNUMBER(H37),ISNUMBER(I37)),I37-H37,"")</f>
-        <v/>
-      </c>
+      <c r="J37" s="8" t="n"/>
       <c r="K37" s="8" t="n"/>
     </row>
     <row r="38">
@@ -1554,10 +1479,7 @@
       <c r="G38" s="8" t="n"/>
       <c r="H38" s="8" t="n"/>
       <c r="I38" s="8" t="n"/>
-      <c r="J38" s="8">
-        <f>IF(AND(ISNUMBER(H38),ISNUMBER(I38)),I38-H38,"")</f>
-        <v/>
-      </c>
+      <c r="J38" s="8" t="n"/>
       <c r="K38" s="8" t="n"/>
     </row>
     <row r="39">
@@ -1569,10 +1491,7 @@
       <c r="G39" s="8" t="n"/>
       <c r="H39" s="8" t="n"/>
       <c r="I39" s="8" t="n"/>
-      <c r="J39" s="8">
-        <f>IF(AND(ISNUMBER(H39),ISNUMBER(I39)),I39-H39,"")</f>
-        <v/>
-      </c>
+      <c r="J39" s="8" t="n"/>
       <c r="K39" s="8" t="n"/>
     </row>
     <row r="40">
@@ -1584,10 +1503,7 @@
       <c r="G40" s="8" t="n"/>
       <c r="H40" s="8" t="n"/>
       <c r="I40" s="8" t="n"/>
-      <c r="J40" s="8">
-        <f>IF(AND(ISNUMBER(H40),ISNUMBER(I40)),I40-H40,"")</f>
-        <v/>
-      </c>
+      <c r="J40" s="8" t="n"/>
       <c r="K40" s="8" t="n"/>
     </row>
     <row r="41">
@@ -1599,10 +1515,7 @@
       <c r="G41" s="8" t="n"/>
       <c r="H41" s="8" t="n"/>
       <c r="I41" s="8" t="n"/>
-      <c r="J41" s="8">
-        <f>IF(AND(ISNUMBER(H41),ISNUMBER(I41)),I41-H41,"")</f>
-        <v/>
-      </c>
+      <c r="J41" s="8" t="n"/>
       <c r="K41" s="8" t="n"/>
     </row>
     <row r="42">
@@ -1614,10 +1527,7 @@
       <c r="G42" s="8" t="n"/>
       <c r="H42" s="8" t="n"/>
       <c r="I42" s="8" t="n"/>
-      <c r="J42" s="8">
-        <f>IF(AND(ISNUMBER(H42),ISNUMBER(I42)),I42-H42,"")</f>
-        <v/>
-      </c>
+      <c r="J42" s="8" t="n"/>
       <c r="K42" s="8" t="n"/>
     </row>
     <row r="43">
@@ -1629,10 +1539,7 @@
       <c r="G43" s="8" t="n"/>
       <c r="H43" s="8" t="n"/>
       <c r="I43" s="8" t="n"/>
-      <c r="J43" s="8">
-        <f>IF(AND(ISNUMBER(H43),ISNUMBER(I43)),I43-H43,"")</f>
-        <v/>
-      </c>
+      <c r="J43" s="8" t="n"/>
       <c r="K43" s="8" t="n"/>
     </row>
     <row r="44">
@@ -1644,10 +1551,7 @@
       <c r="G44" s="8" t="n"/>
       <c r="H44" s="8" t="n"/>
       <c r="I44" s="8" t="n"/>
-      <c r="J44" s="8">
-        <f>IF(AND(ISNUMBER(H44),ISNUMBER(I44)),I44-H44,"")</f>
-        <v/>
-      </c>
+      <c r="J44" s="8" t="n"/>
       <c r="K44" s="8" t="n"/>
     </row>
     <row r="45">
@@ -1659,10 +1563,7 @@
       <c r="G45" s="8" t="n"/>
       <c r="H45" s="8" t="n"/>
       <c r="I45" s="8" t="n"/>
-      <c r="J45" s="8">
-        <f>IF(AND(ISNUMBER(H45),ISNUMBER(I45)),I45-H45,"")</f>
-        <v/>
-      </c>
+      <c r="J45" s="8" t="n"/>
       <c r="K45" s="8" t="n"/>
     </row>
     <row r="46">
@@ -1674,10 +1575,7 @@
       <c r="G46" s="8" t="n"/>
       <c r="H46" s="8" t="n"/>
       <c r="I46" s="8" t="n"/>
-      <c r="J46" s="8">
-        <f>IF(AND(ISNUMBER(H46),ISNUMBER(I46)),I46-H46,"")</f>
-        <v/>
-      </c>
+      <c r="J46" s="8" t="n"/>
       <c r="K46" s="8" t="n"/>
     </row>
     <row r="47">
@@ -1689,10 +1587,7 @@
       <c r="G47" s="8" t="n"/>
       <c r="H47" s="8" t="n"/>
       <c r="I47" s="8" t="n"/>
-      <c r="J47" s="8">
-        <f>IF(AND(ISNUMBER(H47),ISNUMBER(I47)),I47-H47,"")</f>
-        <v/>
-      </c>
+      <c r="J47" s="8" t="n"/>
       <c r="K47" s="8" t="n"/>
     </row>
     <row r="48">
@@ -1704,10 +1599,7 @@
       <c r="G48" s="8" t="n"/>
       <c r="H48" s="8" t="n"/>
       <c r="I48" s="8" t="n"/>
-      <c r="J48" s="8">
-        <f>IF(AND(ISNUMBER(H48),ISNUMBER(I48)),I48-H48,"")</f>
-        <v/>
-      </c>
+      <c r="J48" s="8" t="n"/>
       <c r="K48" s="8" t="n"/>
     </row>
     <row r="49">
@@ -1719,10 +1611,7 @@
       <c r="G49" s="8" t="n"/>
       <c r="H49" s="8" t="n"/>
       <c r="I49" s="8" t="n"/>
-      <c r="J49" s="8">
-        <f>IF(AND(ISNUMBER(H49),ISNUMBER(I49)),I49-H49,"")</f>
-        <v/>
-      </c>
+      <c r="J49" s="8" t="n"/>
       <c r="K49" s="8" t="n"/>
     </row>
     <row r="50">
@@ -1734,10 +1623,7 @@
       <c r="G50" s="8" t="n"/>
       <c r="H50" s="8" t="n"/>
       <c r="I50" s="8" t="n"/>
-      <c r="J50" s="8">
-        <f>IF(AND(ISNUMBER(H50),ISNUMBER(I50)),I50-H50,"")</f>
-        <v/>
-      </c>
+      <c r="J50" s="8" t="n"/>
       <c r="K50" s="8" t="n"/>
     </row>
     <row r="51">
@@ -1749,10 +1635,7 @@
       <c r="G51" s="8" t="n"/>
       <c r="H51" s="8" t="n"/>
       <c r="I51" s="8" t="n"/>
-      <c r="J51" s="8">
-        <f>IF(AND(ISNUMBER(H51),ISNUMBER(I51)),I51-H51,"")</f>
-        <v/>
-      </c>
+      <c r="J51" s="8" t="n"/>
       <c r="K51" s="8" t="n"/>
     </row>
     <row r="52">
@@ -1764,10 +1647,7 @@
       <c r="G52" s="8" t="n"/>
       <c r="H52" s="8" t="n"/>
       <c r="I52" s="8" t="n"/>
-      <c r="J52" s="8">
-        <f>IF(AND(ISNUMBER(H52),ISNUMBER(I52)),I52-H52,"")</f>
-        <v/>
-      </c>
+      <c r="J52" s="8" t="n"/>
       <c r="K52" s="8" t="n"/>
     </row>
     <row r="53">
@@ -1779,10 +1659,7 @@
       <c r="G53" s="8" t="n"/>
       <c r="H53" s="8" t="n"/>
       <c r="I53" s="8" t="n"/>
-      <c r="J53" s="8">
-        <f>IF(AND(ISNUMBER(H53),ISNUMBER(I53)),I53-H53,"")</f>
-        <v/>
-      </c>
+      <c r="J53" s="8" t="n"/>
       <c r="K53" s="8" t="n"/>
     </row>
     <row r="54">
@@ -1794,10 +1671,7 @@
       <c r="G54" s="8" t="n"/>
       <c r="H54" s="8" t="n"/>
       <c r="I54" s="8" t="n"/>
-      <c r="J54" s="8">
-        <f>IF(AND(ISNUMBER(H54),ISNUMBER(I54)),I54-H54,"")</f>
-        <v/>
-      </c>
+      <c r="J54" s="8" t="n"/>
       <c r="K54" s="8" t="n"/>
     </row>
     <row r="55">
@@ -1809,10 +1683,7 @@
       <c r="G55" s="8" t="n"/>
       <c r="H55" s="8" t="n"/>
       <c r="I55" s="8" t="n"/>
-      <c r="J55" s="8">
-        <f>IF(AND(ISNUMBER(H55),ISNUMBER(I55)),I55-H55,"")</f>
-        <v/>
-      </c>
+      <c r="J55" s="8" t="n"/>
       <c r="K55" s="8" t="n"/>
     </row>
     <row r="56">
@@ -1824,10 +1695,7 @@
       <c r="G56" s="8" t="n"/>
       <c r="H56" s="8" t="n"/>
       <c r="I56" s="8" t="n"/>
-      <c r="J56" s="8">
-        <f>IF(AND(ISNUMBER(H56),ISNUMBER(I56)),I56-H56,"")</f>
-        <v/>
-      </c>
+      <c r="J56" s="8" t="n"/>
       <c r="K56" s="8" t="n"/>
     </row>
     <row r="57">
@@ -1839,10 +1707,7 @@
       <c r="G57" s="8" t="n"/>
       <c r="H57" s="8" t="n"/>
       <c r="I57" s="8" t="n"/>
-      <c r="J57" s="8">
-        <f>IF(AND(ISNUMBER(H57),ISNUMBER(I57)),I57-H57,"")</f>
-        <v/>
-      </c>
+      <c r="J57" s="8" t="n"/>
       <c r="K57" s="8" t="n"/>
     </row>
     <row r="58">
@@ -1854,10 +1719,7 @@
       <c r="G58" s="8" t="n"/>
       <c r="H58" s="8" t="n"/>
       <c r="I58" s="8" t="n"/>
-      <c r="J58" s="8">
-        <f>IF(AND(ISNUMBER(H58),ISNUMBER(I58)),I58-H58,"")</f>
-        <v/>
-      </c>
+      <c r="J58" s="8" t="n"/>
       <c r="K58" s="8" t="n"/>
     </row>
     <row r="59">
@@ -1869,10 +1731,7 @@
       <c r="G59" s="8" t="n"/>
       <c r="H59" s="8" t="n"/>
       <c r="I59" s="8" t="n"/>
-      <c r="J59" s="8">
-        <f>IF(AND(ISNUMBER(H59),ISNUMBER(I59)),I59-H59,"")</f>
-        <v/>
-      </c>
+      <c r="J59" s="8" t="n"/>
       <c r="K59" s="8" t="n"/>
     </row>
     <row r="60">
@@ -1884,10 +1743,7 @@
       <c r="G60" s="8" t="n"/>
       <c r="H60" s="8" t="n"/>
       <c r="I60" s="8" t="n"/>
-      <c r="J60" s="8">
-        <f>IF(AND(ISNUMBER(H60),ISNUMBER(I60)),I60-H60,"")</f>
-        <v/>
-      </c>
+      <c r="J60" s="8" t="n"/>
       <c r="K60" s="8" t="n"/>
     </row>
     <row r="61">
@@ -1899,10 +1755,7 @@
       <c r="G61" s="8" t="n"/>
       <c r="H61" s="8" t="n"/>
       <c r="I61" s="8" t="n"/>
-      <c r="J61" s="8">
-        <f>IF(AND(ISNUMBER(H61),ISNUMBER(I61)),I61-H61,"")</f>
-        <v/>
-      </c>
+      <c r="J61" s="8" t="n"/>
       <c r="K61" s="8" t="n"/>
     </row>
     <row r="62">
@@ -1914,10 +1767,7 @@
       <c r="G62" s="8" t="n"/>
       <c r="H62" s="8" t="n"/>
       <c r="I62" s="8" t="n"/>
-      <c r="J62" s="8">
-        <f>IF(AND(ISNUMBER(H62),ISNUMBER(I62)),I62-H62,"")</f>
-        <v/>
-      </c>
+      <c r="J62" s="8" t="n"/>
       <c r="K62" s="8" t="n"/>
     </row>
     <row r="63">
@@ -1929,10 +1779,7 @@
       <c r="G63" s="8" t="n"/>
       <c r="H63" s="8" t="n"/>
       <c r="I63" s="8" t="n"/>
-      <c r="J63" s="8">
-        <f>IF(AND(ISNUMBER(H63),ISNUMBER(I63)),I63-H63,"")</f>
-        <v/>
-      </c>
+      <c r="J63" s="8" t="n"/>
       <c r="K63" s="8" t="n"/>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Pattern tracker: drop stale Low/Med/High dropdown on Anti-Pattern column (left over from pre-Category layout); add Yes/Partial/No dropdown on Tool-detected-fix column
</commit_message>
<xml_diff>
--- a/pattern-tracker.xlsx
+++ b/pattern-tracker.xlsx
@@ -1784,15 +1784,15 @@
     </row>
   </sheetData>
   <dataValidations count="3">
-    <dataValidation sqref="E2:E1000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Low,Med,High"</formula1>
-    </dataValidation>
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Top level,Concepts,API,SDKs,Guides,Operations,Reference,External,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Med,High"</formula1>
     </dataValidation>
+    <dataValidation sqref="H2:H200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Yes,Partial,No"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Add 3 site-level issues (#17 llms.txt+robots+sitemap, #18 head metadata, #19 JSON-LD) — closes audit-tool gap on Discoverability + Structured Data; update README count and tracker dropdown
</commit_message>
<xml_diff>
--- a/pattern-tracker.xlsx
+++ b/pattern-tracker.xlsx
@@ -533,7 +533,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A54"/>
+  <dimension ref="A1:A58"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
@@ -845,22 +845,51 @@
         </is>
       </c>
     </row>
+    <row r="51">
+      <c r="A51" s="11" t="inlineStr">
+        <is>
+          <t>Site-level (audit tool flagged these as missing)</t>
+        </is>
+      </c>
+    </row>
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>Repo: https://github.com/wtd-quillship-demo/quillship-docs</t>
+          <t xml:space="preserve">  #17  llms.txt + robots.txt + sitemap.xml at repo root</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>Live site to audit: https://wtd-quillship-demo.github.io/quillship-docs/</t>
+          <t xml:space="preserve">  #18  HTML head metadata: OpenGraph, canonical URL, markdown alternate link</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  #19  Structured data: JSON-LD TechArticle + BreadcrumbList in layout</t>
+        </is>
+      </c>
+    </row>
+    <row r="55"/>
+    <row r="56">
+      <c r="A56" t="inlineStr">
+        <is>
+          <t>Repo: https://github.com/wtd-quillship-demo/quillship-docs</t>
+        </is>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57" t="inlineStr">
+        <is>
+          <t>Live site to audit: https://wtd-quillship-demo.github.io/quillship-docs/</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" t="inlineStr">
         <is>
           <t>Canonical fix criteria: https://github.com/wtd-quillship-demo/quillship-docs/blob/main/CONTRIBUTING.md#what-ai-readiness-means-here-canonical-list</t>
         </is>
@@ -1785,7 +1814,7 @@
   </sheetData>
   <dataValidations count="3">
     <dataValidation sqref="C2:C200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
-      <formula1>"Top level,Concepts,API,SDKs,Guides,Operations,Reference,External,Other"</formula1>
+      <formula1>"Site-level,Top level,Concepts,API,SDKs,Guides,Operations,Reference,External,Other"</formula1>
     </dataValidation>
     <dataValidation sqref="F2:F200" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Low,Med,High"</formula1>

</xml_diff>